<commit_message>
Refresh neotree_data_keys/ and neotree_scripts/, rebuild dictionaries (v1.2.3)
A three-way sync audit (local/DSH/github) found this repo's own copies of
the web-editor data-key export and script metadata had gone stale
independently of the packaged dictionaries -- rebuilding from this repo's
own inputs would have produced 14 of 18 dictionaries differently from what
is actually shipped. Refreshed both input folders from the internal build
and rebuilt all 36 dictionary files (base + _enriched); content-verified
full parity against the internal build. No previously-shipped dictionary
content has changed -- this closes a latent divergence risk for future
rebuilds, it is not a correction to the current release.

See CHANGELOG.md for details.
</commit_message>
<xml_diff>
--- a/cleaning_pipeline_R/neotree_scripts/mwi-scripts/Generic PHC Admission Bua - metadata.xlsx
+++ b/cleaning_pipeline_R/neotree_scripts/mwi-scripts/Generic PHC Admission Bua - metadata.xlsx
@@ -524,7 +524,7 @@
         <v>$WellvsSick !== 'Norm'</v>
       </c>
       <c r="S2" t="str">
-        <v>{"screenId":"e55b2ca9-a2e7-4ef9-8442-d249588f6bfb","position":9}</v>
+        <v>{"screenId":"c2de1ddb-1a5e-4b65-bd7d-37f650af5a5d","position":9}</v>
       </c>
       <c r="T2" t="str">
         <v/>
@@ -592,7 +592,7 @@
         <v>$MatHIVStat = 'NR'</v>
       </c>
       <c r="S3" t="str">
-        <v>{"screenId":"c9e1fe1d-7300-4155-95e8-77f8be15c701","position":5}</v>
+        <v>{"screenId":"d31d633b-312e-40ca-8106-ff5a2e2367f3","position":5}</v>
       </c>
       <c r="T3" t="str">
         <v/>
@@ -660,7 +660,7 @@
         <v>$MatHIVStat = 'NR'</v>
       </c>
       <c r="S4" t="str">
-        <v>{"screenId":"c9e1fe1d-7300-4155-95e8-77f8be15c701","position":5}</v>
+        <v>{"screenId":"d31d633b-312e-40ca-8106-ff5a2e2367f3","position":5}</v>
       </c>
       <c r="T4" t="str">
         <v/>
@@ -728,7 +728,7 @@
         <v>$MatHIVStat = 'NR'</v>
       </c>
       <c r="S5" t="str">
-        <v>{"screenId":"c9e1fe1d-7300-4155-95e8-77f8be15c701","position":5}</v>
+        <v>{"screenId":"d31d633b-312e-40ca-8106-ff5a2e2367f3","position":5}</v>
       </c>
       <c r="T5" t="str">
         <v/>
@@ -796,7 +796,7 @@
         <v>$MatHIVStat = 'NR'</v>
       </c>
       <c r="S6" t="str">
-        <v>{"screenId":"c9e1fe1d-7300-4155-95e8-77f8be15c701","position":5}</v>
+        <v>{"screenId":"d31d633b-312e-40ca-8106-ff5a2e2367f3","position":5}</v>
       </c>
       <c r="T6" t="str">
         <v/>
@@ -864,7 +864,7 @@
         <v>$MatHIVStat = 'NR'</v>
       </c>
       <c r="S7" t="str">
-        <v>{"screenId":"c9e1fe1d-7300-4155-95e8-77f8be15c701","position":5}</v>
+        <v>{"screenId":"d31d633b-312e-40ca-8106-ff5a2e2367f3","position":5}</v>
       </c>
       <c r="T7" t="str">
         <v/>
@@ -932,7 +932,7 @@
         <v>$MatHIVStat = 'NR'</v>
       </c>
       <c r="S8" t="str">
-        <v>{"screenId":"c9e1fe1d-7300-4155-95e8-77f8be15c701","position":5}</v>
+        <v>{"screenId":"d31d633b-312e-40ca-8106-ff5a2e2367f3","position":5}</v>
       </c>
       <c r="T8" t="str">
         <v/>
@@ -1000,7 +1000,7 @@
         <v>$MatHIVStat = 'NR'</v>
       </c>
       <c r="S9" t="str">
-        <v>{"screenId":"c9e1fe1d-7300-4155-95e8-77f8be15c701","position":5}</v>
+        <v>{"screenId":"d31d633b-312e-40ca-8106-ff5a2e2367f3","position":5}</v>
       </c>
       <c r="T9" t="str">
         <v/>
@@ -1068,7 +1068,7 @@
         <v>$MatHIVStat = 'NR'</v>
       </c>
       <c r="S10" t="str">
-        <v>{"screenId":"c9e1fe1d-7300-4155-95e8-77f8be15c701","position":5}</v>
+        <v>{"screenId":"d31d633b-312e-40ca-8106-ff5a2e2367f3","position":5}</v>
       </c>
       <c r="T10" t="str">
         <v/>
@@ -1136,7 +1136,7 @@
         <v>$MatHIVStat = 'NR'</v>
       </c>
       <c r="S11" t="str">
-        <v>{"screenId":"c9e1fe1d-7300-4155-95e8-77f8be15c701","position":5}</v>
+        <v>{"screenId":"d31d633b-312e-40ca-8106-ff5a2e2367f3","position":5}</v>
       </c>
       <c r="T11" t="str">
         <v/>
@@ -1180,7 +1180,7 @@
         <v/>
       </c>
       <c r="K12" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="L12" t="str">
         <v>No</v>
@@ -1204,7 +1204,7 @@
         <v>$MatHIVStat = 'NR'</v>
       </c>
       <c r="S12" t="str">
-        <v>{"screenId":"c9e1fe1d-7300-4155-95e8-77f8be15c701","position":5}</v>
+        <v>{"screenId":"d31d633b-312e-40ca-8106-ff5a2e2367f3","position":5}</v>
       </c>
       <c r="T12" t="str">
         <v/>
@@ -1408,7 +1408,7 @@
         <v>$Temperature &lt; 36.5</v>
       </c>
       <c r="S15" t="str">
-        <v>{"screenId":"469f4490-b572-4226-afa3-2f4f249f8429","position":8}</v>
+        <v>{"screenId":"22bc0756-7f49-4fd4-8917-5ecfb8a07883","position":8}</v>
       </c>
       <c r="T15" t="str">
         <v/>
@@ -1544,7 +1544,7 @@
         <v>$NeotreeOutcome = 'AdmPNW'</v>
       </c>
       <c r="S17" t="str">
-        <v>{"screenId":"98082b21-f3ee-4c16-b6ea-a9425d52ee85","position":162}</v>
+        <v>{"screenId":"12d91e78-ad08-4bd7-9c5d-dfa677654c6e","position":163}</v>
       </c>
       <c r="T17" t="str">
         <v/>
@@ -1825,7 +1825,7 @@
         <v/>
       </c>
       <c r="V21" t="str">
-        <v>{"actionText":"RESUSCITATION","contentText":"","infoText":"","title":"EMERGENCY MANAGEMENT ","title1":"Resuscitate the baby:","title2":"How to use Bag-Valve-Mask:","title3":"When stable continue with NeoTree","title4":"","text1":"","text2":"","text3":"If no HR for &gt; 10 minutes or remains &lt; 60/min for 20 mins STOP resuscitating but CONTINUE with NeoTree","instructions":"","instructions2":"","instructions3":"","instructions4":"","notes":"","refKey":"","images":{"contentTextImage":null,"image1":{"data":"https://webeditor.neotree.org/files/1be556fa-70c2-48bd-ab8e-1c503400cb93?height=1076&amp;width=588","fileId":"1be556fa-70c2-48bd-ab8e-1c503400cb93","filename":"HBB action plan.jpg","size":"84101"},"image2":{"data":"https://webeditor.neotree.org/files/e0bc71a2-edf0-4759-a58c-b8753e15b6c8?height=312&amp;width=320","fileId":"e0bc71a2-edf0-4759-a58c-b8753e15b6c8","filename":"BVMblue.png","size":"89015"},"image3":{"data":"https://webeditor.neotree.org/files/a836bf2f-e179-440b-bb0c-87b8028266de?height=431&amp;width=447","fileId":"a836bf2f-e179-440b-bb0c-87b8028266de","filename":"Screen Shot 2016-04-22 at 10.26.33.png","size":"108712"}}}</v>
+        <v>{"actionText":"RESUSCITATION","contentText":"","infoText":"","title":"EMERGENCY MANAGEMENT ","title1":"Resuscitate the baby:","title2":"How to use Bag-Valve-Mask:","title3":"When stable continue with NeoTree","title4":"","text1":"","text2":"","text3":"If no HR for &gt; 10 minutes or remains &lt; 60/min for 20 mins STOP resuscitating but CONTINUE with NeoTree","instructions":"","instructions2":"","instructions3":"","instructions4":"","notes":"","refKey":"","images":{"contentTextImage":null,"image1":{"data":"https://webeditor.neotree.org/files/1be556fa-70c2-48bd-ab8e-1c503400cb93?height=1076&amp;width=588","fileId":"1be556fa-70c2-48bd-ab8e-1c503400cb93","filename":"HBB action plan.jpg","size":"84101"},"image2":{"data":"https://webeditor.neotree.org/files/e0bc71a2-edf0-4759-a58c-b8753e15b6c8?height=312&amp;type=png&amp;width=320","fileId":"e0bc71a2-edf0-4759-a58c-b8753e15b6c8","filename":"BVMblue.png","size":"89015"},"image3":{"data":"https://webeditor.neotree.org/files/a836bf2f-e179-440b-bb0c-87b8028266de?height=431&amp;width=447","fileId":"a836bf2f-e179-440b-bb0c-87b8028266de","filename":"Screen Shot 2016-04-22 at 10.26.33.png","size":"108712"}}}</v>
       </c>
     </row>
     <row r="22">
@@ -2277,7 +2277,7 @@
         <v/>
       </c>
       <c r="N28" t="str">
-        <v>[{"value":"Cold","valueLabel":"Trunk feels cold","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"PrCRT","valueLabel":"Capillary Refill Time more than 3 seconds ","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"Wkpulse","valueLabel":"Weak or fast femoral pulses","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"Norm","valueLabel":"NONE","disabledOtherOptionsIfSelected":true,"forbidWIth":[]}]</v>
+        <v>[{"value":"Cold","valueLabel":"Trunk feels cold","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"PrCRT","valueLabel":"Capillary Refill Time more than 3 seconds ","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"Wkpulse","valueLabel":"Weak or fast, thready femoral pulses","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"Norm","valueLabel":"NONE","disabledOtherOptionsIfSelected":true,"forbidWIth":[]}]</v>
       </c>
       <c r="O28" t="str">
         <v/>
@@ -2788,10 +2788,10 @@
         <v>Bua Primary Health Centre</v>
       </c>
       <c r="C36" t="str">
-        <v>Referral Instructions (O2)</v>
+        <v xml:space="preserve">EMERGENCY MANAGEMENT </v>
       </c>
       <c r="D36" t="str">
-        <v>Emergency</v>
+        <v xml:space="preserve">Severe Resp Distress 2 </v>
       </c>
       <c r="E36" t="str">
         <v>management</v>
@@ -2845,7 +2845,7 @@
         <v/>
       </c>
       <c r="V36" t="str">
-        <v>{"actionText":"Referral with Oxygen if available","contentText":"Prepare this baby for referral according to instructions below.\n\nKeep the baby on oxygen if available\nIf oxygen is NOT available CALL referral hospital immediately for guidance and if possible send the baby with accompanying health worker with bag valve mask (BVM) ventilation equipment.\n\nContinue with the Neotree examination.","infoText":"","title":"Referral Instructions (O2)","title1":"Stabilisation","title2":"Communication &amp; Documentation","title3":"Management in Transit","title4":"","text1":"1. Assess ABCCCD (Airway, Breathing, Circulation, Coma, Convulsions and Dehydration) and treat emergency signs \n2. Ensure baby is on Oxygen IF AVAILABLE \n3. Keep Warm - place hat and wrap baby\n4. Review by senior clinician or nurse - if available\n5. Give stat doses of antibiotics - Xpen and Gentamicin\n6. If mum is able to express encourage feeding by cup ONLY if baby can tolerate","text2":"1. Inform receiving facility (KDH) of case summary by phone call or Whatsapp group - discuss availability of portable oxygen &amp; medical escort\n2. Communicate to guardian intention to refer and reasons\n3. Attach Neotree print out ready for transit\n4. Attach all relevant documents/ notes/ checks (glucose, HIV, VDRL etc.)\n","text3":"1. Put baby on portable oxygen IF AVAILABLE\n2. Refer in KMC position unless clinical conditions require observation &amp; care in transit\n3. Refer with escort (Nurse or clinician) with BVM equipment - IF AVAILABLE\n4. Nurse or clinician to bring emergency supplies in ambulance (bag &amp; mask, penguin sucker, dextrose etc.)\n5. IN PERSON handover by nurse or clinician at receiving facility - if possible","instructions":"","instructions2":"","instructions3":"","instructions4":"","notes":"","refKey":"","images":{"contentTextImage":null,"image1":null,"image2":null,"image3":null}}</v>
+        <v>{"actionText":"Severe respiratory distress ","contentText":"If not already on oxygen","infoText":"","title":"EMERGENCY MANAGEMENT ","title1":"1. Airway ","title2":"2. Respiratory support","title3":"3. Feeding support ","title4":"","text1":"- Suction if visible secretions\n- Neutral position (as shown below)","text2":"- Put on oxygen via nasal prongs\n- Maintain Sats 90-95%","text3":"- May need NGT, OGT or IV fluids at a higher level facility\n(Likely to need IV access &amp; antibiotics)\n\n- This baby will need referral to a higher level facility (e.g. KDH or KCH) as will be unable to effectively breast or cup feed","instructions":"","instructions2":"","instructions3":"","instructions4":"","notes":"","refKey":"","images":{"contentTextImage":null,"image1":{"data":"https://webeditor.neotree.org/files/0e1463dd-a7a1-44c6-80f4-feceab769582?height=1044&amp;width=1802","fileId":"0e1463dd-a7a1-44c6-80f4-feceab769582","filename":"0e1463dd-a7a1-44c6-80f4-feceab769582__442b604d-8afc-4e97-8491-13eba0707999.jpeg?w=1802&amp;h=1044","size":199006,"contentType":"image/jpeg"},"image2":{"data":"https://webeditor.neotree.org/files/f6ba4241-8d31-4018-8c2b-5fb647c814fc?height=452&amp;width=514","fileId":"f6ba4241-8d31-4018-8c2b-5fb647c814fc","filename":"f6ba4241-8d31-4018-8c2b-5fb647c814fc__b85885ca-34ef-475c-bc55-a80c7a9b0502.png?w=514&amp;h=452","size":172101,"contentType":"image/png"},"image3":null}}</v>
       </c>
     </row>
     <row r="37">
@@ -2856,10 +2856,10 @@
         <v>Bua Primary Health Centre</v>
       </c>
       <c r="C37" t="str">
-        <v xml:space="preserve">EMERGENCY MANAGEMENT </v>
+        <v>Referral Instructions (O2)</v>
       </c>
       <c r="D37" t="str">
-        <v xml:space="preserve">Severe Resp Distress 2 </v>
+        <v>Emergency</v>
       </c>
       <c r="E37" t="str">
         <v>management</v>
@@ -2913,7 +2913,7 @@
         <v/>
       </c>
       <c r="V37" t="str">
-        <v>{"actionText":"Severe respiratory distress ","contentText":"If not already on oxygen","infoText":"","title":"EMERGENCY MANAGEMENT ","title1":"1. Airway ","title2":"2. Respiratory support","title3":"3. Feeding support ","title4":"","text1":"- Suction if visible secretions\n- Neutral position (as shown below)","text2":"- Put on oxygen via nasal prongs\n- Maintain Sats 90-95%","text3":"- May need NGT, OGT or IV fluids at a higher level facility\n(Likely to need IV access &amp; antibiotics)\n\n- This baby will need referral to a higher level facility (e.g. KDH or KCH) as will be unable to effectively breast or cup feed","instructions":"","instructions2":"","instructions3":"","instructions4":"","notes":"","refKey":"","images":{"contentTextImage":null,"image1":{"data":"https://webeditor.neotree.org/files/0e1463dd-a7a1-44c6-80f4-feceab769582?height=1044&amp;width=1802","fileId":"0e1463dd-a7a1-44c6-80f4-feceab769582","filename":"0e1463dd-a7a1-44c6-80f4-feceab769582__442b604d-8afc-4e97-8491-13eba0707999.jpeg?w=1802&amp;h=1044","size":199006,"contentType":"image/jpeg"},"image2":{"data":"https://webeditor.neotree.org/files/f6ba4241-8d31-4018-8c2b-5fb647c814fc?height=452&amp;width=514","fileId":"f6ba4241-8d31-4018-8c2b-5fb647c814fc","filename":"f6ba4241-8d31-4018-8c2b-5fb647c814fc__b85885ca-34ef-475c-bc55-a80c7a9b0502.png?w=514&amp;h=452","size":172101,"contentType":"image/png"},"image3":null}}</v>
+        <v>{"actionText":"Referral with Oxygen if available","contentText":"Prepare this baby for referral according to instructions below.\n\nKeep the baby on oxygen if available\nIf oxygen is NOT available CALL referral hospital immediately for guidance and if possible send the baby with accompanying health worker with bag valve mask (BVM) ventilation equipment.\n\nContinue with the Neotree examination.","infoText":"","title":"Referral Instructions (O2)","title1":"Stabilisation","title2":"Communication &amp; Documentation","title3":"Management in Transit","title4":"","text1":"1. Assess ABCCCD (Airway, Breathing, Circulation, Coma, Convulsions and Dehydration) and treat emergency signs \n2. Ensure baby is on Oxygen IF AVAILABLE \n3. Keep Warm - place hat and wrap baby\n4. Review by senior clinician or nurse - if available\n5. Give stat doses of antibiotics - Xpen and Gentamicin\n6. If mum is able to express encourage feeding by cup ONLY if baby can tolerate","text2":"1. Inform receiving facility (KDH) of case summary by phone call or Whatsapp group - discuss availability of portable oxygen &amp; medical escort\n2. Communicate to guardian intention to refer and reasons\n3. Attach Neotree print out ready for transit\n4. Attach all relevant documents/ notes/ checks (glucose, HIV, VDRL etc.)\n","text3":"1. Put baby on portable oxygen IF AVAILABLE\n2. Refer in KMC position unless clinical conditions require observation &amp; care in transit\n3. Refer with escort (Nurse or clinician) with BVM equipment - IF AVAILABLE\n4. Nurse or clinician to bring emergency supplies in ambulance (bag &amp; mask, penguin sucker, dextrose etc.)\n5. IN PERSON handover by nurse or clinician at receiving facility - if possible","instructions":"","instructions2":"","instructions3":"","instructions4":"","notes":"","refKey":"","images":{"contentTextImage":null,"image1":null,"image2":null,"image3":null}}</v>
       </c>
     </row>
     <row r="38">
@@ -6655,7 +6655,7 @@
         <v/>
       </c>
       <c r="V92" t="str">
-        <v>{"actionText":"Assessment of tone","contentText":"Weigh the baby completely naked. While you do this:\n\n1. Check the tone as below\n2. Check the spine for spina bifida \n3. Measure the head circumference\n","infoText":"","title":"Tone","title1":"A = normal, B = hypotonic","title2":"","title3":"","title4":"","text1":"","text2":"","text3":"","instructions":"","instructions2":"","instructions3":"","instructions4":"","notes":"","refKey":"","images":{"contentTextImage":null,"image1":{"data":"https://webeditor.neotree.org/files/84cc2d14-a505-4cb9-ad01-af2bafe8c72c?height=810&amp;width=716","fileId":"84cc2d14-a505-4cb9-ad01-af2bafe8c72c","filename":"Tone jpeg.jpg","size":"133387"},"image2":null,"image3":null}}</v>
+        <v>{"actionText":"Assessment of tone","contentText":"Weigh the baby completely naked. While you do this:\n\n1. Check the tone as below\n2. Check the spine for spina bifida \n3. Measure the head circumference\n","infoText":"","title":"Tone","title1":"A = normal, B = hypotonic","title2":"","title3":"","title4":"","text1":"","text2":"","text3":"","instructions":"","instructions2":"","instructions3":"","instructions4":"","notes":"","refKey":"","images":{"contentTextImage":null,"image1":{"data":"https://webeditor.neotree.org/files/84cc2d14-a505-4cb9-ad01-af2bafe8c72c?height=810&amp;orientation=1&amp;type=jpg&amp;width=716","fileId":"84cc2d14-a505-4cb9-ad01-af2bafe8c72c","filename":"Tone jpeg.jpg","size":"133387"},"image2":null,"image3":null}}</v>
       </c>
     </row>
     <row r="93">
@@ -6927,7 +6927,7 @@
         <v/>
       </c>
       <c r="V96" t="str">
-        <v>{"actionText":"THOMPSON SCORE","contentText":"Please complete Thompson score for BA / HIE by assessing posture, moro and grasp as shown below\n","infoText":"","title":"THOMPSON SCORE","title1":"Posture","title2":"","title3":"THOMPSON SCORE (fill in on next page)","title4":"","text1":"","text2":"","text3":"","instructions":"","instructions2":"","instructions3":"","instructions4":"","notes":"","refKey":"","images":{"contentTextImage":null,"image1":{"data":"https://webeditor.neotree.org/files/fbcf627f-4f91-4f4d-b4a5-9751d44e2e20?height=732&amp;width=1058","fileId":"fbcf627f-4f91-4f4d-b4a5-9751d44e2e20","filename":"Posture jpeg.jpg","size":"200569"},"image2":{"data":"https://webeditor.neotree.org/files/f01bde99-8f6b-41f0-a69d-1453ff4e36f0?height=608&amp;width=942","fileId":"f01bde99-8f6b-41f0-a69d-1453ff4e36f0","filename":"Morograsp jpeg.jpg","size":"187244"},"image3":{"data":"https://webeditor.neotree.org/files/4670ebdb-2fd4-435b-a0c7-f012441d0038?height=652&amp;width=1148","fileId":"4670ebdb-2fd4-435b-a0c7-f012441d0038","filename":"Thompson jpeg.jpg","size":"179793"}}}</v>
+        <v>{"actionText":"THOMPSON SCORE","contentText":"Please complete Thompson score for BA / HIE by assessing posture, moro and grasp as shown below\n","infoText":"","title":"THOMPSON SCORE","title1":"Posture","title2":"","title3":"THOMPSON SCORE (fill in on next page)","title4":"","text1":"","text2":"","text3":"","instructions":"","instructions2":"","instructions3":"","instructions4":"","notes":"","refKey":"","images":{"contentTextImage":null,"image1":{"data":"https://webeditor.neotree.org/files/fbcf627f-4f91-4f4d-b4a5-9751d44e2e20?height=732&amp;orientation=1&amp;type=jpg&amp;width=1058","fileId":"fbcf627f-4f91-4f4d-b4a5-9751d44e2e20","filename":"Posture jpeg.jpg","size":"200569"},"image2":{"data":"https://webeditor.neotree.org/files/f01bde99-8f6b-41f0-a69d-1453ff4e36f0?height=608&amp;orientation=1&amp;type=jpg&amp;width=942","fileId":"f01bde99-8f6b-41f0-a69d-1453ff4e36f0","filename":"Morograsp jpeg.jpg","size":"187244"},"image3":{"data":"https://webeditor.neotree.org/files/4670ebdb-2fd4-435b-a0c7-f012441d0038?height=652&amp;orientation=1&amp;type=jpg&amp;width=1148","fileId":"4670ebdb-2fd4-435b-a0c7-f012441d0038","filename":"Thompson jpeg.jpg","size":"179793"}}}</v>
       </c>
     </row>
     <row r="97">
@@ -8239,7 +8239,7 @@
         <v>multi_select</v>
       </c>
       <c r="F116" t="str">
-        <v>SignsDehydrations</v>
+        <v>DehydraSigns</v>
       </c>
       <c r="G116" t="str">
         <v>Signs of Dehydration</v>
@@ -8263,7 +8263,7 @@
         <v>$AgeA = 'N' or ($AgeCat = 'NB48' or $AgeCat = 'INF72' or $AgeCat = 'INF')</v>
       </c>
       <c r="N116" t="str">
-        <v>[{"value":"PSP","valueLabel":"Prolonged skin pinch","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"DMM","valueLabel":"Dry Mucous Membranes ","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"SE","valueLabel":"Sunken Eyes","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"Norm","valueLabel":"NONE","disabledOtherOptionsIfSelected":true,"forbidWIth":[]}]</v>
+        <v>[{"value":"PSP","valueLabel":"Prolonged skin pinch ( &gt; 2seconds)","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"DMM","valueLabel":"Dry Mucous Membranes ","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"SE","valueLabel":"Sunken Eyes","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"Norm","valueLabel":"NONE","disabledOtherOptionsIfSelected":true,"forbidWIth":[]}]</v>
       </c>
       <c r="O116" t="str">
         <v>$AgeA = 'N' or ($AgeCat = 'NB48' or $AgeCat = 'INF72' or $AgeCat = 'INF')</v>
@@ -9419,7 +9419,7 @@
         <v/>
       </c>
       <c r="N133" t="str">
-        <v>[{"value":"DIB","valueLabel":"Fast or laboured breathing","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"NBr","valueLabel":"Noisy Breathing ","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"Cough","valueLabel":"Cough","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"Apn","valueLabel":"Apnoea","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"BE","valueLabel":"Blue episodes ","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"Gasp","valueLabel":"Gasping","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"Norm","valueLabel":"NONE","disabledOtherOptionsIfSelected":true,"forbidWIth":[]}]</v>
+        <v>[{"value":"DIB","valueLabel":"Fast or laboured breathing","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"NBr","valueLabel":"Noisy Breathing ","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"Cough","valueLabel":"Cough","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"Apn","valueLabel":"Apnea","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"BE","valueLabel":"Blue episodes ","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"Gasp","valueLabel":"Gasping","disabledOtherOptionsIfSelected":false,"forbidWIth":[]},{"value":"Norm","valueLabel":"NONE","disabledOtherOptionsIfSelected":true,"forbidWIth":[]}]</v>
       </c>
       <c r="O133" t="str">
         <v/>
@@ -10350,7 +10350,7 @@
         <v>ReferredFrom</v>
       </c>
       <c r="G147" t="str">
-        <v>Name of Referring Facility</v>
+        <v>Name of referring Facility</v>
       </c>
       <c r="H147" t="str">
         <v>dropdown</v>
@@ -10371,7 +10371,7 @@
         <v>$InOrOut = 'Out' and $ReferredFrom2 = 'F'</v>
       </c>
       <c r="N147" t="str">
-        <v>[{"value":"AncF","valueLabel":"Anchor Farm"},{"value":"Cha","valueLabel":"Chambwe"},{"value":"Chm","valueLabel":"Chamwabvi"},{"value":"Chi","valueLabel":"Chilanga"},{"value":"Chn","valueLabel":"Chinyama"},{"value":"Chu","valueLabel":"Chulu"},{"value":"Gog","valueLabel":"Gogode"},{"value":"Kak","valueLabel":"Kakwale"},{"value":"KAL","valueLabel":"Kaluluma Health Centre"},{"value":"Kam","valueLabel":"Kamboni"},{"value":"Kap","valueLabel":"Kapelula"},{"value":"Kai","valueLabel":"Kapichira"},{"value":"Kay","valueLabel":"Kapyanga"},{"value":"Kaw","valueLabel":"Kawamba"},{"value":"Kho","valueLabel":"Khola"},{"value":"Lin","valueLabel":"Linyangwa"},{"value":"Liv","valueLabel":"Livwezi"},{"value":"Lod","valueLabel":"Lodjwa"},{"value":"Mdu","valueLabel":"Mdunga"},{"value":"Mkh","valueLabel":"Mkhota"},{"value":"Mny","valueLabel":"Mnyanja"},{"value":"Mpe","valueLabel":"Mpepa"},{"value":"Mtu","valueLabel":"Mtunthama"},{"value":"Mzi","valueLabel":"Mziza"},{"value":"New","valueLabel":"Newa"},{"value":"Nkh","valueLabel":"Nkhamenya"},{"value":"Ofe","valueLabel":"Ofesi"},{"value":"San","valueLabel":"Santhe"},{"value":"Sim","valueLabel":"Simlemba"},{"value":"StA","valueLabel":"St Andrew’s"},{"value":"StD","valueLabel":"St Dennis"},{"value":"StF","valueLabel":"St Faith"},{"value":"Wim","valueLabel":"Wimbe"},{"value":"O","valueLabel":"Other"}]</v>
+        <v>[{"value":"AncF","valueLabel":"Anchor Farm"},{"value":"Cha","valueLabel":"Chambwe"},{"value":"Chi","valueLabel":"Chilanga"},{"value":"Chn","valueLabel":"Chinyama"},{"value":"Gog","valueLabel":"Gogode"},{"value":"Kak","valueLabel":"Kakwale"},{"value":"KAL","valueLabel":"Kaluluma Health Centre"},{"value":"Kai","valueLabel":"Kapichira"},{"value":"Kay","valueLabel":"Kapyanga"},{"value":"Kho","valueLabel":"Khola"},{"value":"Lin","valueLabel":"Linyangwa"},{"value":"Liv","valueLabel":"Livwezi"},{"value":"Lod","valueLabel":"Lodjwa"},{"value":"Mdu","valueLabel":"Mdunga"},{"value":"Mkh","valueLabel":"Mkhota"},{"value":"Mny","valueLabel":"Mnyanja"},{"value":"Mtu","valueLabel":"Mtunthama"},{"value":"Mzi","valueLabel":"Mziza"},{"value":"New","valueLabel":"Newa"},{"value":"Nkh","valueLabel":"Nkhamenya"},{"value":"Ofe","valueLabel":"Ofesi"},{"value":"StA","valueLabel":"St Andrew’s"},{"value":"StD","valueLabel":"St Dennis"},{"value":"StF","valueLabel":"St Faith"},{"value":"Wim","valueLabel":"Wimbe"},{"value":"Bua","valueLabel":"Bua Health Centre"},{"value":"CHV","valueLabel":"Chamwabvi Health Centre"},{"value":"CHL","valueLabel":"Chulu Health Centre"},{"value":"KBM","valueLabel":"Kamboni Health Centre"},{"value":"KPL","valueLabel":"Kapelula Health Centre"},{"value":"KWB","valueLabel":"Kawamba Health Centre"},{"value":"MPP","valueLabel":"Mpepa Health Centre"},{"value":"SAN","valueLabel":"Santhe Health Centre"},{"value":"SLB","valueLabel":"Simlemba Health Centre"},{"value":"O","valueLabel":"Other"}]</v>
       </c>
       <c r="O147" t="str">
         <v/>
@@ -10643,7 +10643,7 @@
         <v>$PlaceBirth = 'Hosp' or $PlaceBirth = 'HC'</v>
       </c>
       <c r="N151" t="str">
-        <v>[{"value":"AncF","valueLabel":"Anchor Farm"},{"value":"Cha","valueLabel":"Chambwe"},{"value":"Chm","valueLabel":"Chamwabvi"},{"value":"Chi","valueLabel":"Chilanga"},{"value":"Chn","valueLabel":"Chinyama"},{"value":"Chu","valueLabel":"Chulu"},{"value":"Gog","valueLabel":"Gogode"},{"value":"Kak","valueLabel":"Kakwale"},{"value":"KAL","valueLabel":"Kaluluma Health Centre"},{"value":"Kam","valueLabel":"Kamboni"},{"value":"Kap","valueLabel":"Kapelula"},{"value":"Kai","valueLabel":"Kapichira"},{"value":"Kay","valueLabel":"Kapyanga"},{"value":"Kaw","valueLabel":"Kawamba"},{"value":"Kdh","valueLabel":"Kasungu District Hospital"},{"value":"Kho","valueLabel":"Khola"},{"value":"Lin","valueLabel":"Linyangwa"},{"value":"Liv","valueLabel":"Livwezi"},{"value":"Lod","valueLabel":"Lodjwa"},{"value":"Mdu","valueLabel":"Mdunga"},{"value":"Mkh","valueLabel":"Mkhota"},{"value":"Mny","valueLabel":"Mnyanja"},{"value":"Mpe","valueLabel":"Mpepa"},{"value":"Mtu","valueLabel":"Mtunthama"},{"value":"Mzi","valueLabel":"Mziza"},{"value":"New","valueLabel":"Newa"},{"value":"Nkh","valueLabel":"Nkhamenya"},{"value":"Ofe","valueLabel":"Ofesi"},{"value":"San","valueLabel":"Santhe"},{"value":"Sim","valueLabel":"Simlemba"},{"value":"StA","valueLabel":"St Andrew’s"},{"value":"StD","valueLabel":"St Dennis"},{"value":"StF","valueLabel":"St Faith"},{"value":"Wim","valueLabel":"Wimbe"},{"value":"O","valueLabel":"Other"}]</v>
+        <v>[{"value":"AncF","valueLabel":"Anchor Farm"},{"value":"Cha","valueLabel":"Chambwe"},{"value":"Chi","valueLabel":"Chilanga"},{"value":"Chn","valueLabel":"Chinyama"},{"value":"Gog","valueLabel":"Gogode"},{"value":"Kak","valueLabel":"Kakwale"},{"value":"KAL","valueLabel":"Kaluluma Health Centre"},{"value":"Kai","valueLabel":"Kapichira"},{"value":"Kay","valueLabel":"Kapyanga"},{"value":"Kdh","valueLabel":"Kasungu District Hospital"},{"value":"Kho","valueLabel":"Khola"},{"value":"Lin","valueLabel":"Linyangwa"},{"value":"Liv","valueLabel":"Livwezi"},{"value":"Lod","valueLabel":"Lodjwa"},{"value":"Mdu","valueLabel":"Mdunga"},{"value":"Mkh","valueLabel":"Mkhota"},{"value":"Mny","valueLabel":"Mnyanja"},{"value":"Mtu","valueLabel":"Mtunthama"},{"value":"Mzi","valueLabel":"Mziza"},{"value":"New","valueLabel":"Newa"},{"value":"Nkh","valueLabel":"Nkhamenya"},{"value":"Ofe","valueLabel":"Ofesi"},{"value":"StA","valueLabel":"St Andrew’s"},{"value":"StD","valueLabel":"St Dennis"},{"value":"StF","valueLabel":"St Faith"},{"value":"Wim","valueLabel":"Wimbe"},{"value":"CHL","valueLabel":"Chulu Health Centre"},{"value":"Bua","valueLabel":"Bua"},{"value":"CHV","valueLabel":"Chamwabvi Health Centre"},{"value":"KBM","valueLabel":"Kamboni Health Centre"},{"value":"KPL","valueLabel":"Kapelula Health Centre"},{"value":"KWB","valueLabel":"Kawamba Health Centre"},{"value":"MPP","valueLabel":"Mpepa Health Centre"},{"value":"SAN","valueLabel":"Santhe Health Centre"},{"value":"SLB","valueLabel":"Simlemba Health Centre"},{"value":"O","valueLabel":"Other"}]</v>
       </c>
       <c r="O151" t="str">
         <v/>
@@ -12062,10 +12062,10 @@
         <v/>
       </c>
       <c r="K172" t="str">
+        <v>No</v>
+      </c>
+      <c r="L172" t="str">
         <v>Yes</v>
-      </c>
-      <c r="L172" t="str">
-        <v>No</v>
       </c>
       <c r="M172" t="str">
         <v/>
@@ -12186,7 +12186,7 @@
         <v>HIVtestResult</v>
       </c>
       <c r="G174" t="str">
-        <v>What was the Result?</v>
+        <v xml:space="preserve">What was the Result? </v>
       </c>
       <c r="H174" t="str">
         <v>dropdown</v>
@@ -12198,7 +12198,7 @@
         <v/>
       </c>
       <c r="K174" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="L174" t="str">
         <v>No</v>
@@ -12266,7 +12266,7 @@
         <v/>
       </c>
       <c r="K175" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="L175" t="str">
         <v>No</v>
@@ -12334,7 +12334,7 @@
         <v/>
       </c>
       <c r="K176" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="L176" t="str">
         <v>No</v>
@@ -15906,7 +15906,7 @@
         <v/>
       </c>
     </row>
-    <row r="229">
+    <row r="229" xml:space="preserve">
       <c r="A229" t="str">
         <v>Generic PHC Admission</v>
       </c>
@@ -15949,8 +15949,9 @@
       <c r="N229" t="str">
         <v/>
       </c>
-      <c r="O229" t="str">
-        <v>$RefDia = 'RD' or $RefDia = 'BA'</v>
+      <c r="O229" t="str" xml:space="preserve">
+        <v xml:space="preserve">$RefDia = 'RD'
+$RefDia = 'BA'</v>
       </c>
       <c r="P229" t="str">
         <v/>
@@ -16110,7 +16111,7 @@
         <v>{"actionText":" Referral for Abdominal surgical management ","contentText":"These babies need stabilisation PRIOR to transfer  - this significantly improves their outcome\n\nAim to leave and transfer this baby within an hour!","infoText":"","title":"Referral Instructions - Diagnoses requiring Abdominal surgical management ","title1":"Stabilisation","title2":"Antibiotics &amp; Management (in transit)","title3":"Communication &amp; Documentation","title4":"","text1":"1. Assess Airway, breathing, circulation and manage any emergency signs \n2. Keep baby warm - place hat and wrap baby \n3. Wrap bowel in clingfilm or sterile bag up to armpit - to minimise fluid loss\n4. Nil By Mouth and insert NGT for aspiration on free drainage\n5. Insert cannula and give 20 mL/kg of normal saline or Hartmann’s solution as a bolus\n6. Start IV Fluids at 60mls/kg/day  - 10% Dextrose\n7. Monitor blood sugar","text2":"1. Start antibiotics\n           Ceftriaxone (50mg/kg) once daily\n           Metronidazole (15mg/kg as a single loading dose, followed by 7.5mg/kg every 12hr starting 24 hr after the loading dose)\n2. Transfer in KMC unless clinical conditions require observation &amp; care in transit\n3. Refer with escort (Nurse or clinician) - IF AVAILABLE\n4. Nurse or clinician to bring emergency supplies in ambulance (bag &amp; mask, penguin sucker, dextrose etc.)\n5. IN PERSON handover at receiving facility - if possible \n\n","text3":"1. Inform receiving facility (KDH or KCH) of case summary by phone - discuss availability of medical escort\n2. Communicate to guardian intention to refer and reasons - Counsel and educate parents - encourage parental bonding\n3. Attach Neotree print out ready for transfer\n4. Attach all relevant documents/ notes/ checks (glucose, HIV, VDRL etc.)\n\n\n\n\n*Please complete the section below by hand*\n\nTime Ambulance called ________________ am/pm\n\nTime Ambulance arrived ________________ am/pm ","instructions":"","instructions2":"","instructions3":"","instructions4":"","notes":"","refKey":"$RefDia = 'AbdoSurg'","images":{"contentTextImage":null,"image1":null,"image2":null,"image3":null}}</v>
       </c>
     </row>
-    <row r="232">
+    <row r="232" xml:space="preserve">
       <c r="A232" t="str">
         <v>Generic PHC Admission</v>
       </c>
@@ -16153,8 +16154,13 @@
       <c r="N232" t="str">
         <v/>
       </c>
-      <c r="O232" t="str">
-        <v>$RefDia = 'VExLBW' or $RefDia = 'LBWsick' or $RefDia = 'Conv' or $RefDia = 'NSep' or $RefDia = 'Jaun' or $RefDia = 'Cong'</v>
+      <c r="O232" t="str" xml:space="preserve">
+        <v xml:space="preserve">$RefDia = 'VExLBW'
+$RefDia = 'LBWsick'
+$RefDia = 'Conv'
+$RefDia = 'NSep'
+$RefDia = 'Jaun'
+$RefDia = 'Cong'</v>
       </c>
       <c r="P232" t="str">
         <v/>
@@ -17785,7 +17791,7 @@
         <v>Possible Meconium Aspiration</v>
       </c>
       <c r="H2" t="str">
-        <v>2932</v>
+        <v>3244</v>
       </c>
       <c r="I2" t="str">
         <v>editor</v>
@@ -17874,7 +17880,7 @@
         <v>Suspected Neonatal Sepsis</v>
       </c>
       <c r="H3" t="str">
-        <v>2933</v>
+        <v>3245</v>
       </c>
       <c r="I3" t="str">
         <v>editor</v>
@@ -17963,7 +17969,7 @@
         <v>Difficulty Feeding</v>
       </c>
       <c r="H4" t="str">
-        <v>2934</v>
+        <v>3246</v>
       </c>
       <c r="I4" t="str">
         <v>editor</v>
@@ -18043,7 +18049,7 @@
         <v>Dehydration</v>
       </c>
       <c r="H5" t="str">
-        <v>2935</v>
+        <v>3247</v>
       </c>
       <c r="I5" t="str">
         <v>editor</v>
@@ -18058,7 +18064,7 @@
         <v/>
       </c>
       <c r="M5" t="str">
-        <v>[{"expression":"$SignsDehydrations = 'PSP'","name":"Prolonged skin pinch","type":"sign","weight":"1.0","position":1,"symptomId":"0a180cff-303a-4c03-8b56-43b0105b91af","printable":true,"keyId":"9159f93f-1dac-4343-bcdb-35db47569ade"},{"expression":"$SignsDehydrations = 'DMM'","name":"Dry Mucous Membranes ","type":"sign","weight":"1.0","position":2,"symptomId":"ce994d42-b614-40d7-b3e1-038e772e0afa","printable":true,"keyId":"c73e08c5-a5bf-4bae-8904-a0503b76d184"},{"expression":"$SignsDehydrations = 'SE'","name":"Sunken eyes","type":"sign","weight":"1.0","position":3,"symptomId":"ce7e2d95-0257-4aa1-a04e-f83689e3dc07","printable":true,"keyId":"026555d2-aba2-461d-b56e-86ac13ee4121"},{"expression":"$Fontanelle = 'Sunk'","name":"Fontanelle Sunken","type":"sign","weight":"1.0","position":4,"symptomId":"d655b4de-34f4-4799-8306-b84d5c625cff","printable":true,"keyId":"f8725ec4-2fdb-49d5-bf56-935d73a6115d"}]</v>
+        <v>[{"expression":"$SignsDehydrations = 'PSP'","name":"Prolonged skin pinch","type":"sign","weight":"1.0","position":1,"symptomId":"0a180cff-303a-4c03-8b56-43b0105b91af","printable":true,"keyId":"9159f93f-1dac-4343-bcdb-35db47569ade"},{"expression":"$SignsDehydrations = 'DMM'","name":"Dry Mucous Membranes ","type":"sign","weight":"1.0","position":2,"symptomId":"ce994d42-b614-40d7-b3e1-038e772e0afa","printable":true,"keyId":"c73e08c5-a5bf-4bae-8904-a0503b76d184"},{"expression":"$SignsDehydrations = 'SE'","name":"Sunken eyes","type":"sign","weight":"1.0","position":3,"symptomId":"ce7e2d95-0257-4aa1-a04e-f83689e3dc07","printable":true,"keyId":"026555d2-aba2-461d-b56e-86ac13ee4121"},{"expression":"$Fontanelle = 'Sunk'","name":"Sunken Fontanelle","type":"sign","weight":"1.0","position":4,"symptomId":"d655b4de-34f4-4799-8306-b84d5c625cff","printable":true,"key":"SunkFont"}]</v>
       </c>
       <c r="N5" t="str">
         <v xml:space="preserve">Refer to WHO plan A, B or C as below: </v>
@@ -18120,7 +18126,7 @@
         <v>Congenital Heart Disease</v>
       </c>
       <c r="H6" t="str">
-        <v>2936</v>
+        <v>3248</v>
       </c>
       <c r="I6" t="str">
         <v/>
@@ -18206,7 +18212,7 @@
         <v>Anaemia</v>
       </c>
       <c r="H7" t="str">
-        <v>2937</v>
+        <v>3249</v>
       </c>
       <c r="I7" t="str">
         <v>editor</v>
@@ -18291,7 +18297,7 @@
         <v>Congenital Abnormality</v>
       </c>
       <c r="H8" t="str">
-        <v>2938</v>
+        <v>3250</v>
       </c>
       <c r="I8" t="str">
         <v>editor</v>
@@ -18377,7 +18383,7 @@
         <v>Pneumonia / Bronchiolitis</v>
       </c>
       <c r="H9" t="str">
-        <v>2939</v>
+        <v>3251</v>
       </c>
       <c r="I9" t="str">
         <v>editor</v>
@@ -18462,7 +18468,7 @@
         <v>Transient Tachypnoea of Newborn (TTN)</v>
       </c>
       <c r="H10" t="str">
-        <v>2940</v>
+        <v>3252</v>
       </c>
       <c r="I10" t="str">
         <v>editor</v>
@@ -18548,7 +18554,7 @@
         <v>Umbilical Hernia</v>
       </c>
       <c r="H11" t="str">
-        <v>2941</v>
+        <v>3253</v>
       </c>
       <c r="I11" t="str">
         <v>editor</v>
@@ -18625,7 +18631,7 @@
         <v>Meningitis</v>
       </c>
       <c r="H12" t="str">
-        <v>2942</v>
+        <v>3254</v>
       </c>
       <c r="I12" t="str">
         <v>editor</v>
@@ -18702,7 +18708,7 @@
         <v>Ambiguous Genetalia</v>
       </c>
       <c r="H13" t="str">
-        <v>2943</v>
+        <v>3255</v>
       </c>
       <c r="I13" t="str">
         <v>editor</v>
@@ -18779,7 +18785,7 @@
         <v>Untreated Maternal Syphilis</v>
       </c>
       <c r="H14" t="str">
-        <v>2944</v>
+        <v>3256</v>
       </c>
       <c r="I14" t="str">
         <v>editor</v>
@@ -18856,7 +18862,7 @@
         <v>Abdominal obstruction</v>
       </c>
       <c r="H15" t="str">
-        <v>2945</v>
+        <v>3257</v>
       </c>
       <c r="I15" t="str">
         <v>editor</v>
@@ -18933,7 +18939,7 @@
         <v>Birth Trauma</v>
       </c>
       <c r="H16" t="str">
-        <v>2946</v>
+        <v>3258</v>
       </c>
       <c r="I16" t="str">
         <v>editor</v>
@@ -19010,7 +19016,7 @@
         <v>Apnoea of prematurity</v>
       </c>
       <c r="H17" t="str">
-        <v>2947</v>
+        <v>3259</v>
       </c>
       <c r="I17" t="str">
         <v>editor</v>
@@ -19087,7 +19093,7 @@
         <v>Birth Asphyxia</v>
       </c>
       <c r="H18" t="str">
-        <v>2948</v>
+        <v>3260</v>
       </c>
       <c r="I18" t="str">
         <v>editor</v>
@@ -19164,7 +19170,7 @@
         <v>Convulsions</v>
       </c>
       <c r="H19" t="str">
-        <v>2949</v>
+        <v>3261</v>
       </c>
       <c r="I19" t="str">
         <v>editor</v>
@@ -19255,7 +19261,7 @@
         <v>Low Birth Weight (1500-2499g)</v>
       </c>
       <c r="H20" t="str">
-        <v>2950</v>
+        <v>3262</v>
       </c>
       <c r="I20" t="str">
         <v>editor</v>
@@ -19340,7 +19346,7 @@
         <v>Very Low Birth Weight (1000-1499g)</v>
       </c>
       <c r="H21" t="str">
-        <v>2951</v>
+        <v>3263</v>
       </c>
       <c r="I21" t="str">
         <v>editor</v>
@@ -19426,7 +19432,7 @@
         <v>Extremely Low Birth Weight (&lt;1000g)</v>
       </c>
       <c r="H22" t="str">
-        <v>2952</v>
+        <v>3264</v>
       </c>
       <c r="I22" t="str">
         <v>editor</v>
@@ -19511,7 +19517,7 @@
         <v>High Birth Weight (&gt;4000g at birth)</v>
       </c>
       <c r="H23" t="str">
-        <v>2953</v>
+        <v>3265</v>
       </c>
       <c r="I23" t="str">
         <v>editor</v>
@@ -19588,7 +19594,7 @@
         <v>Mild Hypothermia</v>
       </c>
       <c r="H24" t="str">
-        <v>2954</v>
+        <v>3266</v>
       </c>
       <c r="I24" t="str">
         <v>editor</v>
@@ -19673,7 +19679,7 @@
         <v>Moderate Hypothermia</v>
       </c>
       <c r="H25" t="str">
-        <v>2955</v>
+        <v>3267</v>
       </c>
       <c r="I25" t="str">
         <v>editor</v>
@@ -19758,7 +19764,7 @@
         <v>Severe Hypothermia</v>
       </c>
       <c r="H26" t="str">
-        <v>2956</v>
+        <v>3268</v>
       </c>
       <c r="I26" t="str">
         <v>editor</v>
@@ -19843,7 +19849,7 @@
         <v>Hyperthermia</v>
       </c>
       <c r="H27" t="str">
-        <v>2957</v>
+        <v>3269</v>
       </c>
       <c r="I27" t="str">
         <v>editor</v>
@@ -19921,7 +19927,7 @@
         <v>Premature (32-36 weeks)</v>
       </c>
       <c r="H28" t="str">
-        <v>2958</v>
+        <v>3270</v>
       </c>
       <c r="I28" t="str">
         <v>editor</v>
@@ -20015,7 +20021,7 @@
         <v>Very Premature (28-31 weeks)</v>
       </c>
       <c r="H29" t="str">
-        <v>2959</v>
+        <v>3271</v>
       </c>
       <c r="I29" t="str">
         <v>editor</v>
@@ -20109,7 +20115,7 @@
         <v>Extremely Premature (&lt;28 weeks)</v>
       </c>
       <c r="H30" t="str">
-        <v>2960</v>
+        <v>3272</v>
       </c>
       <c r="I30" t="str">
         <v>editor</v>
@@ -20203,7 +20209,7 @@
         <v>Hypoglycaemia (symptomatic)</v>
       </c>
       <c r="H31" t="str">
-        <v>2961</v>
+        <v>3273</v>
       </c>
       <c r="I31" t="str">
         <v>editor</v>
@@ -20285,7 +20291,7 @@
         <v>Hypoglycaemia (NOT symptomatic)</v>
       </c>
       <c r="H32" t="str">
-        <v>2962</v>
+        <v>3274</v>
       </c>
       <c r="I32" t="str">
         <v>editor</v>
@@ -20364,7 +20370,7 @@
         <v>At Risk of Hypoglycaemia</v>
       </c>
       <c r="H33" t="str">
-        <v>2963</v>
+        <v>3275</v>
       </c>
       <c r="I33" t="str">
         <v/>
@@ -20456,7 +20462,7 @@
         <v>HIV Unknown</v>
       </c>
       <c r="H34" t="str">
-        <v>2964</v>
+        <v>3276</v>
       </c>
       <c r="I34" t="str">
         <v/>
@@ -20545,7 +20551,7 @@
         <v>HIV Low Risk</v>
       </c>
       <c r="H35" t="str">
-        <v>2965</v>
+        <v>3277</v>
       </c>
       <c r="I35" t="str">
         <v/>
@@ -20628,7 +20634,7 @@
         <v>HIV High Risk</v>
       </c>
       <c r="H36" t="str">
-        <v>2966</v>
+        <v>3278</v>
       </c>
       <c r="I36" t="str">
         <v/>
@@ -20716,7 +20722,7 @@
         <v>Physiological Jaundice</v>
       </c>
       <c r="H37" t="str">
-        <v>2967</v>
+        <v>3279</v>
       </c>
       <c r="I37" t="str">
         <v>editor</v>
@@ -20745,7 +20751,7 @@
         <v xml:space="preserve">3. Educate parents on how to monitor for jaundice </v>
       </c>
       <c r="Q37" t="str">
-        <v>{"data":"https://webeditor.neotree.org/files/361b5b75-8599-415a-b25d-f4586c3dbe8c?height=446&amp;width=642","fileId":"361b5b75-8599-415a-b25d-f4586c3dbe8c","filename":"Jaundice.png","size":"127149"}</v>
+        <v>{"data":"https://webeditor.neotree.org/files/361b5b75-8599-415a-b25d-f4586c3dbe8c?height=446&amp;type=png&amp;width=642","fileId":"361b5b75-8599-415a-b25d-f4586c3dbe8c","filename":"Jaundice.png","size":"127149"}</v>
       </c>
       <c r="R37" t="str">
         <v>{"data":"https://webeditor.neotree.org/files/9c741b43-cea6-4b95-824b-3f5dc657f0d1?height=550&amp;width=790","fileId":"9c741b43-cea6-4b95-824b-3f5dc657f0d1","filename":"COIN_Jaund2.png","size":"86572"}</v>
@@ -20795,7 +20801,7 @@
         <v>Pathological Jaundice</v>
       </c>
       <c r="H38" t="str">
-        <v>2968</v>
+        <v>3280</v>
       </c>
       <c r="I38" t="str">
         <v/>
@@ -20886,7 +20892,7 @@
         <v>Prolonged Jaundice</v>
       </c>
       <c r="H39" t="str">
-        <v>2969</v>
+        <v>3281</v>
       </c>
       <c r="I39" t="str">
         <v/>
@@ -20967,7 +20973,7 @@
         <v>Hypoxic Ischaemic Encephalopathy</v>
       </c>
       <c r="H40" t="str">
-        <v>2970</v>
+        <v>3282</v>
       </c>
       <c r="I40" t="str">
         <v/>
@@ -21058,7 +21064,7 @@
         <v>Suspected Hypoxic Ischaemic Encephalopathy</v>
       </c>
       <c r="H41" t="str">
-        <v>2971</v>
+        <v>3283</v>
       </c>
       <c r="I41" t="str">
         <v/>
@@ -21149,7 +21155,7 @@
         <v>Prematurity with Respiratory Distress</v>
       </c>
       <c r="H42" t="str">
-        <v>2972</v>
+        <v>3284</v>
       </c>
       <c r="I42" t="str">
         <v>editor</v>
@@ -21244,7 +21250,7 @@
         <v>Term baby with Respiratory Distress</v>
       </c>
       <c r="H43" t="str">
-        <v>2973</v>
+        <v>3285</v>
       </c>
       <c r="I43" t="str">
         <v/>
@@ -21338,7 +21344,7 @@
         <v>Gastroschisis</v>
       </c>
       <c r="H44" t="str">
-        <v>2974</v>
+        <v>3286</v>
       </c>
       <c r="I44" t="str">
         <v/>
@@ -21430,7 +21436,7 @@
         <v>Omphalocele</v>
       </c>
       <c r="H45" t="str">
-        <v>2975</v>
+        <v>3287</v>
       </c>
       <c r="I45" t="str">
         <v/>
@@ -21515,7 +21521,7 @@
         <v>Cleft lip and/or palate with RD</v>
       </c>
       <c r="H46" t="str">
-        <v>2976</v>
+        <v>3288</v>
       </c>
       <c r="I46" t="str">
         <v/>
@@ -21597,7 +21603,7 @@
         <v>Cleft lip</v>
       </c>
       <c r="H47" t="str">
-        <v>2977</v>
+        <v>3289</v>
       </c>
       <c r="I47" t="str">
         <v/>
@@ -21679,7 +21685,7 @@
         <v>Cleft lip and/or palate</v>
       </c>
       <c r="H48" t="str">
-        <v>2978</v>
+        <v>3290</v>
       </c>
       <c r="I48" t="str">
         <v/>
@@ -21765,7 +21771,7 @@
         <v>Myelomeningocele</v>
       </c>
       <c r="H49" t="str">
-        <v>2979</v>
+        <v>3291</v>
       </c>
       <c r="I49" t="str">
         <v/>
@@ -21849,7 +21855,7 @@
         <v>Congenital dislocation of the hip (CDH)</v>
       </c>
       <c r="H50" t="str">
-        <v>2980</v>
+        <v>3292</v>
       </c>
       <c r="I50" t="str">
         <v/>
@@ -21931,7 +21937,7 @@
         <v>Moderate Talipes (club foot)</v>
       </c>
       <c r="H51" t="str">
-        <v>2981</v>
+        <v>3293</v>
       </c>
       <c r="I51" t="str">
         <v/>
@@ -22010,7 +22016,7 @@
         <v>Mild Talipes (club foot)</v>
       </c>
       <c r="H52" t="str">
-        <v>2982</v>
+        <v>3294</v>
       </c>
       <c r="I52" t="str">
         <v/>
@@ -22088,7 +22094,7 @@
         <v>Risk factors for sepsis (Not symptomatic)</v>
       </c>
       <c r="H53" t="str">
-        <v>2983</v>
+        <v>3295</v>
       </c>
       <c r="I53" t="str">
         <v>editor</v>

</xml_diff>